<commit_message>
Add Cassandra and MongoDB distributed test plans
- C-001: Single-node write (cassandra-stress, 50M ops, thread sweep)
- C-002: Single-node read baseline
- C-003: 3-node cluster mixed (RF=3, CL=QUORUM)
- C-004: Cluster scaling 3→6 nodes
- MG-001: Single-node YCSB workload A (50/50 r/w)
- MG-002: Single-node YCSB workload B (95/5 r/w)
- MG-003: 3-node replica set with write concern majority
- MG-004: Sharded cluster scaling (2→4 shards)
</commit_message>
<xml_diff>
--- a/docs/Database_Benchmark_Test_Plan.xlsx
+++ b/docs/Database_Benchmark_Test_Plan.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -890,6 +890,190 @@
       </c>
       <c r="E18" s="4" t="inlineStr"/>
     </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>C-001</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Cassandra Single-Node Write</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr"/>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Requires: Cassandra install on node 103</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>C-002</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Cassandra Single-Node Read</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Depends on: C-001 (dataset)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>C-003</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Cassandra 3-Node Mixed</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr"/>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Requires: Cassandra on 103, 104, 106</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>C-004</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Cassandra Cluster Scaling (3→6)</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr"/>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Requires: Cassandra on all 6 nodes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>MG-001</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>MongoDB Single-Node YCSB-A</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Requires: MongoDB + YCSB install on 103/101</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>MG-002</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>MongoDB Single-Node YCSB-B</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr"/>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Depends on: MG-001 (dataset)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>MG-003</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>MongoDB 3-Node Replica Set</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Requires: MongoDB on 103, 104, 106</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>MG-004</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>MongoDB Sharded Cluster</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr"/>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Requires: Full sharded topology (6 nodes)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -901,7 +1085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1812,6 +1996,438 @@
           <t>PASS</t>
         </is>
       </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>C-001</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Cassandra</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Single-Node Write Throughput</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>cassandra-stress write: sequential inserts, CL=ONE</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>cassandra-stress</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>n=50M, threads=[64,128,256,512], cl=ONE, rf=1, -node 103</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Cassandra 4.x/5.x, single node, 103, default heap 8G</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Stress tool co-located or from node 101</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>Establish single-node write baseline. Target: &gt;200K ops/sec.</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>C-002</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Cassandra</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Single-Node Read Throughput</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>cassandra-stress read: random reads from populated dataset</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>cassandra-stress</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>n=50M (pre-loaded), threads=[64,128,256,512], cl=ONE, rf=1</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Cassandra, single node, 103</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>From node 101</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Establish single-node read baseline. Compare to write throughput.</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr"/>
+      <c r="L21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>C-003</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Cassandra</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>3-Node Cluster Mixed Workload</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>cassandra-stress mixed (r/w=50/50): 3-node ring, RF=3, CL=QUORUM</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>cassandra-stress</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>n=50M, threads=[128,256,512], cl=QUORUM, rf=3, mixed ratio=1:1</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Cassandra 3-node cluster on 103, 104, 106, vnodes=256</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>2 client nodes (101, 102) running stress independently</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>Measure distributed throughput with replication overhead. Compare to single-node.</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr"/>
+      <c r="L22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>C-004</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Cassandra</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Cluster Scaling (3→6 nodes)</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>cassandra-stress mixed: compare 3-node vs 6-node ring at fixed workload</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>cassandra-stress</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>n=50M, threads=256, cl=QUORUM, rf=3</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Cassandra ring: 3-node (103,104,106) then 6-node (+101,102,107)</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>External stress clients as available</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Validate linear throughput scaling with node count. Target: ~2× at 6 nodes.</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr"/>
+      <c r="L23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>MG-001</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>MongoDB</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Single-Node YCSB Workload A</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>YCSB workload A: 50% read, 50% update, Zipfian distribution</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>YCSB (Yahoo Cloud Serving Benchmark)</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>recordcount=50M, operationcount=10M, threads=[64,128,256,512], workload=A</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>mongod 7.x, single node 103, WiredTiger, directoryPerDB</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>YCSB client from node 101</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>Establish MongoDB single-node mixed baseline. Compare to Redis/MySQL.</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr"/>
+      <c r="L24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>MG-002</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>MongoDB</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Single-Node YCSB Workload B (Read-Heavy)</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>YCSB workload B: 95% read, 5% update, Zipfian distribution</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>YCSB</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>recordcount=50M, operationcount=10M, threads=[64,128,256,512], workload=B</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>mongod 7.x, single node 103, WiredTiger</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>YCSB client from node 101</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Measure MongoDB read-dominated performance. Compare to workload A.</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr"/>
+      <c r="L25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>MG-003</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>MongoDB</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>3-Node Replica Set Mixed</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>YCSB workload A against replica set (w=majority, r=primary)</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>YCSB</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>recordcount=50M, operationcount=10M, threads=256, w=majority, readPreference=primary</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>MongoDB 3-node replica set on 103(primary), 104, 106</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>2 YCSB clients (101, 102)</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>Measure replication overhead vs single-node. Target: &lt;30% degradation vs MG-001.</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr"/>
+      <c r="L26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>MG-004</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>MongoDB</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Sharded Cluster Scaling</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>YCSB workload A against sharded cluster (2 shards → 4 shards)</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>YCSB</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>recordcount=100M, operationcount=10M, threads=256, sharded collection (hashed _id)</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>mongos + config servers + 2-4 shard replica sets across nodes 102-107</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>2 YCSB clients (101, available node)</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>Validate horizontal scaling. Target: ~2× throughput at 4 shards vs 2.</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>